<commit_message>
Fix 0% match rate: add column normalization to upload handler, auto-detect Razorpay/Bank column formats, regenerate clean datasets
</commit_message>
<xml_diff>
--- a/reconciliation_report.xlsx
+++ b/reconciliation_report.xlsx
@@ -496,33 +496,33 @@
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>pay_860104ef9b31</t>
+          <t>pay_a6c807b36cb2</t>
         </is>
       </c>
       <c r="C2" s="1" t="inlineStr">
         <is>
-          <t>UTR645003308438</t>
+          <t>UTR50761855847</t>
         </is>
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
-          <t>MERCH_004</t>
+          <t>MERCH_002</t>
         </is>
       </c>
       <c r="E2" s="1" t="n">
-        <v>39245.35</v>
+        <v>43374.32</v>
       </c>
       <c r="F2" s="1" t="n">
-        <v>39245.35</v>
+        <v>43374.32</v>
       </c>
       <c r="G2" s="1" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="H2" s="1" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="I2" s="1" t="n">
@@ -535,7 +535,7 @@
       </c>
       <c r="K2" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -547,33 +547,33 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>pay_cf92979f2c52</t>
+          <t>pay_025214eb3c22</t>
         </is>
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>UTR539573870210</t>
+          <t>UTR67919123398</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>MERCH_001</t>
+          <t>MERCH_005</t>
         </is>
       </c>
       <c r="E3" s="1" t="n">
-        <v>3884.72</v>
+        <v>19486.9</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>3884.72</v>
+        <v>19486.9</v>
       </c>
       <c r="G3" s="1" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="H3" s="1" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="I3" s="1" t="n">
@@ -586,7 +586,7 @@
       </c>
       <c r="K3" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -598,33 +598,33 @@
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>pay_370d4e2ed8da</t>
+          <t>pay_00ebd2269bf4</t>
         </is>
       </c>
       <c r="C4" s="1" t="inlineStr">
         <is>
-          <t>UTR917721496742</t>
+          <t>UTR407930040114</t>
         </is>
       </c>
       <c r="D4" s="1" t="inlineStr">
         <is>
-          <t>MERCH_003</t>
+          <t>MERCH_005</t>
         </is>
       </c>
       <c r="E4" s="1" t="n">
-        <v>18665.36</v>
+        <v>19782.19</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>18665.36</v>
+        <v>19782.19</v>
       </c>
       <c r="G4" s="1" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="H4" s="1" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="I4" s="1" t="n">
@@ -637,7 +637,7 @@
       </c>
       <c r="K4" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -649,33 +649,33 @@
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
-          <t>pay_dafd0c223193</t>
+          <t>pay_1c25ed4d607b</t>
         </is>
       </c>
       <c r="C5" s="1" t="inlineStr">
         <is>
-          <t>UTR917927588086</t>
+          <t>UTR668448685759</t>
         </is>
       </c>
       <c r="D5" s="1" t="inlineStr">
         <is>
-          <t>MERCH_005</t>
+          <t>MERCH_003</t>
         </is>
       </c>
       <c r="E5" s="1" t="n">
-        <v>3386.06</v>
+        <v>20046.72</v>
       </c>
       <c r="F5" s="1" t="n">
-        <v>3386.06</v>
+        <v>20046.72</v>
       </c>
       <c r="G5" s="1" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="H5" s="1" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="I5" s="1" t="n">
@@ -688,7 +688,7 @@
       </c>
       <c r="K5" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -700,33 +700,33 @@
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
-          <t>pay_9f66e0875037</t>
+          <t>pay_b998a268f604</t>
         </is>
       </c>
       <c r="C6" s="1" t="inlineStr">
         <is>
-          <t>UTR496606355719</t>
+          <t>UTR468891916207</t>
         </is>
       </c>
       <c r="D6" s="1" t="inlineStr">
         <is>
-          <t>MERCH_002</t>
+          <t>MERCH_001</t>
         </is>
       </c>
       <c r="E6" s="1" t="n">
-        <v>4553.96</v>
+        <v>10745.51</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>4553.96</v>
+        <v>10745.51</v>
       </c>
       <c r="G6" s="1" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="H6" s="1" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="I6" s="1" t="n">
@@ -739,7 +739,7 @@
       </c>
       <c r="K6" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -751,33 +751,33 @@
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
-          <t>pay_76361ba25642</t>
+          <t>pay_e3d6d02cfa9b</t>
         </is>
       </c>
       <c r="C7" s="1" t="inlineStr">
         <is>
-          <t>UTR537535591814</t>
+          <t>UTR567036584703</t>
         </is>
       </c>
       <c r="D7" s="1" t="inlineStr">
         <is>
-          <t>MERCH_003</t>
+          <t>MERCH_001</t>
         </is>
       </c>
       <c r="E7" s="1" t="n">
-        <v>41296.61</v>
+        <v>40897.38</v>
       </c>
       <c r="F7" s="1" t="n">
-        <v>41296.61</v>
+        <v>40897.38</v>
       </c>
       <c r="G7" s="1" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="H7" s="1" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="I7" s="1" t="n">
@@ -790,7 +790,7 @@
       </c>
       <c r="K7" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -802,12 +802,12 @@
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
-          <t>pay_7111e77acb25</t>
+          <t>pay_d3e1b38848ca</t>
         </is>
       </c>
       <c r="C8" s="1" t="inlineStr">
         <is>
-          <t>UTR585303759910</t>
+          <t>UTR496763033647</t>
         </is>
       </c>
       <c r="D8" s="1" t="inlineStr">
@@ -816,19 +816,19 @@
         </is>
       </c>
       <c r="E8" s="1" t="n">
-        <v>33866.38</v>
+        <v>13130.12</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>33866.38</v>
+        <v>13130.12</v>
       </c>
       <c r="G8" s="1" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="H8" s="1" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="I8" s="1" t="n">
@@ -841,7 +841,7 @@
       </c>
       <c r="K8" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -853,33 +853,33 @@
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
-          <t>pay_1d4d4fcc7ea0</t>
+          <t>pay_3cf1faa18fad</t>
         </is>
       </c>
       <c r="C9" s="1" t="inlineStr">
         <is>
-          <t>UTR686436941263</t>
+          <t>UTR515548139192</t>
         </is>
       </c>
       <c r="D9" s="1" t="inlineStr">
         <is>
-          <t>MERCH_001</t>
+          <t>MERCH_003</t>
         </is>
       </c>
       <c r="E9" s="1" t="n">
-        <v>41341.97</v>
+        <v>29339.69</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>41341.97</v>
+        <v>29339.69</v>
       </c>
       <c r="G9" s="1" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="H9" s="1" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="I9" s="1" t="n">
@@ -892,7 +892,7 @@
       </c>
       <c r="K9" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -904,33 +904,33 @@
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
-          <t>pay_0f6eebe05a8d</t>
+          <t>pay_45cdaae2e843</t>
         </is>
       </c>
       <c r="C10" s="1" t="inlineStr">
         <is>
-          <t>UTR225053106683</t>
+          <t>UTR505323033518</t>
         </is>
       </c>
       <c r="D10" s="1" t="inlineStr">
         <is>
-          <t>MERCH_004</t>
+          <t>MERCH_001</t>
         </is>
       </c>
       <c r="E10" s="1" t="n">
-        <v>27455.33</v>
+        <v>21554.32</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>27455.33</v>
+        <v>21554.32</v>
       </c>
       <c r="G10" s="1" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="H10" s="1" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="I10" s="1" t="n">
@@ -943,7 +943,7 @@
       </c>
       <c r="K10" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -955,12 +955,12 @@
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
-          <t>pay_fde1bd955148</t>
+          <t>pay_e57cc7afabbe</t>
         </is>
       </c>
       <c r="C11" s="1" t="inlineStr">
         <is>
-          <t>UTR46715223012</t>
+          <t>UTR66435399718</t>
         </is>
       </c>
       <c r="D11" s="1" t="inlineStr">
@@ -969,19 +969,19 @@
         </is>
       </c>
       <c r="E11" s="1" t="n">
-        <v>6456</v>
+        <v>21886.68</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>6456</v>
+        <v>21886.68</v>
       </c>
       <c r="G11" s="1" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="H11" s="1" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="I11" s="1" t="n">
@@ -994,7 +994,7 @@
       </c>
       <c r="K11" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -1006,12 +1006,12 @@
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
-          <t>pay_a6308f4c600e</t>
+          <t>pay_fc6a2ac3ddb6</t>
         </is>
       </c>
       <c r="C12" s="1" t="inlineStr">
         <is>
-          <t>UTR339511118944</t>
+          <t>UTR328781285086</t>
         </is>
       </c>
       <c r="D12" s="1" t="inlineStr">
@@ -1020,19 +1020,19 @@
         </is>
       </c>
       <c r="E12" s="1" t="n">
-        <v>41942.64</v>
+        <v>17455.9</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>41942.64</v>
+        <v>17455.9</v>
       </c>
       <c r="G12" s="1" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="H12" s="1" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="I12" s="1" t="n">
@@ -1045,7 +1045,7 @@
       </c>
       <c r="K12" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -1057,33 +1057,33 @@
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
-          <t>pay_3d3a6b301801</t>
+          <t>pay_a740aea66df8</t>
         </is>
       </c>
       <c r="C13" s="1" t="inlineStr">
         <is>
-          <t>UTR124132654229</t>
+          <t>UTR87489678765</t>
         </is>
       </c>
       <c r="D13" s="1" t="inlineStr">
         <is>
-          <t>MERCH_002</t>
+          <t>MERCH_001</t>
         </is>
       </c>
       <c r="E13" s="1" t="n">
-        <v>36152.11</v>
+        <v>24878.89</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>36152.11</v>
+        <v>24878.89</v>
       </c>
       <c r="G13" s="1" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="H13" s="1" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="I13" s="1" t="n">
@@ -1096,7 +1096,7 @@
       </c>
       <c r="K13" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -1108,33 +1108,33 @@
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
-          <t>pay_2ef2b0679151</t>
+          <t>pay_13341603613c</t>
         </is>
       </c>
       <c r="C14" s="1" t="inlineStr">
         <is>
-          <t>UTR923226603670</t>
+          <t>UTR147013145657</t>
         </is>
       </c>
       <c r="D14" s="1" t="inlineStr">
         <is>
-          <t>MERCH_003</t>
+          <t>MERCH_005</t>
         </is>
       </c>
       <c r="E14" s="1" t="n">
-        <v>43993.1</v>
+        <v>26301.37</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>43993.1</v>
+        <v>26301.37</v>
       </c>
       <c r="G14" s="1" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="H14" s="1" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="I14" s="1" t="n">
@@ -1147,7 +1147,7 @@
       </c>
       <c r="K14" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -1159,24 +1159,24 @@
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
-          <t>pay_4d784f85bdb1</t>
+          <t>pay_791f4ce7bb2c</t>
         </is>
       </c>
       <c r="C15" s="1" t="inlineStr">
         <is>
-          <t>UTR821445087274</t>
+          <t>UTR252932759822</t>
         </is>
       </c>
       <c r="D15" s="1" t="inlineStr">
         <is>
-          <t>MERCH_004</t>
+          <t>MERCH_003</t>
         </is>
       </c>
       <c r="E15" s="1" t="n">
-        <v>39744.84</v>
+        <v>34825.02</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>39744.84</v>
+        <v>34825.02</v>
       </c>
       <c r="G15" s="1" t="inlineStr">
         <is>
@@ -1185,7 +1185,7 @@
       </c>
       <c r="H15" s="1" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="I15" s="1" t="n">
@@ -1198,7 +1198,7 @@
       </c>
       <c r="K15" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -1210,33 +1210,33 @@
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
-          <t>pay_f9f3a7b2ac14</t>
+          <t>pay_8ef9a72b3890</t>
         </is>
       </c>
       <c r="C16" s="1" t="inlineStr">
         <is>
-          <t>UTR541978326411</t>
+          <t>UTR640803120467</t>
         </is>
       </c>
       <c r="D16" s="1" t="inlineStr">
         <is>
-          <t>MERCH_001</t>
+          <t>MERCH_004</t>
         </is>
       </c>
       <c r="E16" s="1" t="n">
-        <v>41959.2</v>
+        <v>7252.52</v>
       </c>
       <c r="F16" s="1" t="n">
-        <v>41959.2</v>
+        <v>7252.52</v>
       </c>
       <c r="G16" s="1" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="H16" s="1" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="I16" s="1" t="n">
@@ -1249,7 +1249,7 @@
       </c>
       <c r="K16" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -1261,24 +1261,24 @@
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
-          <t>pay_8730bfe15363</t>
+          <t>pay_cea5ee444320</t>
         </is>
       </c>
       <c r="C17" s="1" t="inlineStr">
         <is>
-          <t>UTR517598383310</t>
+          <t>UTR213834420873</t>
         </is>
       </c>
       <c r="D17" s="1" t="inlineStr">
         <is>
-          <t>MERCH_003</t>
+          <t>MERCH_001</t>
         </is>
       </c>
       <c r="E17" s="1" t="n">
-        <v>28245.91</v>
+        <v>29085.95</v>
       </c>
       <c r="F17" s="1" t="n">
-        <v>28245.91</v>
+        <v>29085.95</v>
       </c>
       <c r="G17" s="1" t="inlineStr">
         <is>
@@ -1300,7 +1300,7 @@
       </c>
       <c r="K17" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -1312,12 +1312,12 @@
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
-          <t>pay_b4d4416d4d1c</t>
+          <t>pay_1f28375bf739</t>
         </is>
       </c>
       <c r="C18" s="1" t="inlineStr">
         <is>
-          <t>UTR709026549699</t>
+          <t>UTR231777934167</t>
         </is>
       </c>
       <c r="D18" s="1" t="inlineStr">
@@ -1326,19 +1326,19 @@
         </is>
       </c>
       <c r="E18" s="1" t="n">
-        <v>32946.76</v>
+        <v>27187.75</v>
       </c>
       <c r="F18" s="1" t="n">
-        <v>32946.76</v>
+        <v>27187.75</v>
       </c>
       <c r="G18" s="1" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="H18" s="1" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="I18" s="1" t="n">
@@ -1351,7 +1351,7 @@
       </c>
       <c r="K18" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -1363,33 +1363,33 @@
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
-          <t>pay_894cc5254c59</t>
+          <t>pay_d83e0cad21e4</t>
         </is>
       </c>
       <c r="C19" s="1" t="inlineStr">
         <is>
-          <t>UTR588048671775</t>
+          <t>UTR868563113084</t>
         </is>
       </c>
       <c r="D19" s="1" t="inlineStr">
         <is>
-          <t>MERCH_001</t>
+          <t>MERCH_005</t>
         </is>
       </c>
       <c r="E19" s="1" t="n">
-        <v>27187.07</v>
+        <v>5572.78</v>
       </c>
       <c r="F19" s="1" t="n">
-        <v>27187.07</v>
+        <v>5572.78</v>
       </c>
       <c r="G19" s="1" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="H19" s="1" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="I19" s="1" t="n">
@@ -1402,7 +1402,7 @@
       </c>
       <c r="K19" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -1414,33 +1414,33 @@
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
-          <t>pay_caa94c213f37</t>
+          <t>pay_116c9fd763d3</t>
         </is>
       </c>
       <c r="C20" s="1" t="inlineStr">
         <is>
-          <t>UTR938323677696</t>
+          <t>UTR974118540399</t>
         </is>
       </c>
       <c r="D20" s="1" t="inlineStr">
         <is>
-          <t>MERCH_003</t>
+          <t>MERCH_001</t>
         </is>
       </c>
       <c r="E20" s="1" t="n">
-        <v>8883.209999999999</v>
+        <v>5381.11</v>
       </c>
       <c r="F20" s="1" t="n">
-        <v>8883.209999999999</v>
+        <v>5381.11</v>
       </c>
       <c r="G20" s="1" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="H20" s="1" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="I20" s="1" t="n">
@@ -1453,7 +1453,7 @@
       </c>
       <c r="K20" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -1465,33 +1465,33 @@
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
-          <t>pay_74f9b3e3473f</t>
+          <t>pay_7b5afcf619df</t>
         </is>
       </c>
       <c r="C21" s="1" t="inlineStr">
         <is>
-          <t>UTR784466177518</t>
+          <t>UTR567406237153</t>
         </is>
       </c>
       <c r="D21" s="1" t="inlineStr">
         <is>
-          <t>MERCH_002</t>
+          <t>MERCH_003</t>
         </is>
       </c>
       <c r="E21" s="1" t="n">
-        <v>20943.5</v>
+        <v>42958.74</v>
       </c>
       <c r="F21" s="1" t="n">
-        <v>20943.5</v>
+        <v>42958.74</v>
       </c>
       <c r="G21" s="1" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="H21" s="1" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="I21" s="1" t="n">
@@ -1504,7 +1504,7 @@
       </c>
       <c r="K21" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -1516,12 +1516,12 @@
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
-          <t>pay_40fa10829cc2</t>
+          <t>pay_4d044be35065</t>
         </is>
       </c>
       <c r="C22" s="1" t="inlineStr">
         <is>
-          <t>UTR391541135666</t>
+          <t>UTR473831951302</t>
         </is>
       </c>
       <c r="D22" s="1" t="inlineStr">
@@ -1530,19 +1530,19 @@
         </is>
       </c>
       <c r="E22" s="1" t="n">
-        <v>24644.79</v>
+        <v>44234.06</v>
       </c>
       <c r="F22" s="1" t="n">
-        <v>24644.79</v>
+        <v>44234.06</v>
       </c>
       <c r="G22" s="1" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="H22" s="1" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="I22" s="1" t="n">
@@ -1555,7 +1555,7 @@
       </c>
       <c r="K22" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -1567,33 +1567,33 @@
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
-          <t>pay_bee23f0c49cd</t>
+          <t>pay_4b97e8e1baf7</t>
         </is>
       </c>
       <c r="C23" s="1" t="inlineStr">
         <is>
-          <t>UTR414768152489</t>
+          <t>UTR672251886946</t>
         </is>
       </c>
       <c r="D23" s="1" t="inlineStr">
         <is>
-          <t>MERCH_002</t>
+          <t>MERCH_005</t>
         </is>
       </c>
       <c r="E23" s="1" t="n">
-        <v>12745.26</v>
+        <v>22704.89</v>
       </c>
       <c r="F23" s="1" t="n">
-        <v>12745.26</v>
+        <v>22704.89</v>
       </c>
       <c r="G23" s="1" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="H23" s="1" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="I23" s="1" t="n">
@@ -1606,7 +1606,7 @@
       </c>
       <c r="K23" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -1618,12 +1618,12 @@
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
-          <t>pay_4ed503ce3557</t>
+          <t>pay_a223c29644ab</t>
         </is>
       </c>
       <c r="C24" s="1" t="inlineStr">
         <is>
-          <t>UTR12584043189</t>
+          <t>UTR838785969577</t>
         </is>
       </c>
       <c r="D24" s="1" t="inlineStr">
@@ -1632,19 +1632,19 @@
         </is>
       </c>
       <c r="E24" s="1" t="n">
-        <v>28178.84</v>
+        <v>27015.77</v>
       </c>
       <c r="F24" s="1" t="n">
-        <v>28178.84</v>
+        <v>27015.77</v>
       </c>
       <c r="G24" s="1" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="H24" s="1" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="I24" s="1" t="n">
@@ -1657,7 +1657,7 @@
       </c>
       <c r="K24" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -1669,33 +1669,33 @@
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
-          <t>pay_8e8864caa9e6</t>
+          <t>pay_6f410e703393</t>
         </is>
       </c>
       <c r="C25" s="1" t="inlineStr">
         <is>
-          <t>UTR67792957294</t>
+          <t>UTR327793776008</t>
         </is>
       </c>
       <c r="D25" s="1" t="inlineStr">
         <is>
-          <t>MERCH_004</t>
+          <t>MERCH_001</t>
         </is>
       </c>
       <c r="E25" s="1" t="n">
-        <v>23287.05</v>
+        <v>22431.65</v>
       </c>
       <c r="F25" s="1" t="n">
-        <v>23287.05</v>
+        <v>22431.65</v>
       </c>
       <c r="G25" s="1" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="H25" s="1" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="I25" s="1" t="n">
@@ -1708,7 +1708,7 @@
       </c>
       <c r="K25" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -1720,33 +1720,33 @@
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
-          <t>pay_b5ef09bd0eb0</t>
+          <t>pay_4a98862afc90</t>
         </is>
       </c>
       <c r="C26" s="1" t="inlineStr">
         <is>
-          <t>UTR408249077235</t>
+          <t>UTR9975251818</t>
         </is>
       </c>
       <c r="D26" s="1" t="inlineStr">
         <is>
-          <t>MERCH_005</t>
+          <t>MERCH_002</t>
         </is>
       </c>
       <c r="E26" s="1" t="n">
-        <v>5703.79</v>
+        <v>25591.01</v>
       </c>
       <c r="F26" s="1" t="n">
-        <v>5703.79</v>
+        <v>25591.01</v>
       </c>
       <c r="G26" s="1" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="H26" s="1" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I26" s="1" t="n">
@@ -1759,7 +1759,7 @@
       </c>
       <c r="K26" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -1771,33 +1771,33 @@
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
-          <t>pay_b0acdd0d5ae8</t>
+          <t>pay_1318853c5616</t>
         </is>
       </c>
       <c r="C27" s="1" t="inlineStr">
         <is>
-          <t>UTR878270854638</t>
+          <t>UTR191478285140</t>
         </is>
       </c>
       <c r="D27" s="1" t="inlineStr">
         <is>
-          <t>MERCH_004</t>
+          <t>MERCH_003</t>
         </is>
       </c>
       <c r="E27" s="1" t="n">
-        <v>38482.22</v>
+        <v>12740.44</v>
       </c>
       <c r="F27" s="1" t="n">
-        <v>38482.22</v>
+        <v>12740.44</v>
       </c>
       <c r="G27" s="1" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="H27" s="1" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="I27" s="1" t="n">
@@ -1810,7 +1810,7 @@
       </c>
       <c r="K27" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -1822,33 +1822,33 @@
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
-          <t>pay_19954a2e836f</t>
+          <t>pay_416c1639d0b9</t>
         </is>
       </c>
       <c r="C28" s="1" t="inlineStr">
         <is>
-          <t>UTR612666029665</t>
+          <t>UTR884439879230</t>
         </is>
       </c>
       <c r="D28" s="1" t="inlineStr">
         <is>
-          <t>MERCH_001</t>
+          <t>MERCH_003</t>
         </is>
       </c>
       <c r="E28" s="1" t="n">
-        <v>16282.82</v>
+        <v>30288.66</v>
       </c>
       <c r="F28" s="1" t="n">
-        <v>16282.82</v>
+        <v>30288.66</v>
       </c>
       <c r="G28" s="1" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="H28" s="1" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="I28" s="1" t="n">
@@ -1861,7 +1861,7 @@
       </c>
       <c r="K28" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -1873,33 +1873,33 @@
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
-          <t>pay_9c3a12b8301a</t>
+          <t>pay_fe91606cbeb6</t>
         </is>
       </c>
       <c r="C29" s="1" t="inlineStr">
         <is>
-          <t>UTR825523379507</t>
+          <t>UTR236077545067</t>
         </is>
       </c>
       <c r="D29" s="1" t="inlineStr">
         <is>
-          <t>MERCH_001</t>
+          <t>MERCH_004</t>
         </is>
       </c>
       <c r="E29" s="1" t="n">
-        <v>36108.11</v>
+        <v>20790.07</v>
       </c>
       <c r="F29" s="1" t="n">
-        <v>36108.11</v>
+        <v>20790.07</v>
       </c>
       <c r="G29" s="1" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="H29" s="1" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="I29" s="1" t="n">
@@ -1912,7 +1912,7 @@
       </c>
       <c r="K29" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -1924,33 +1924,33 @@
       </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
-          <t>pay_212540c84172</t>
+          <t>pay_98df1b10c79f</t>
         </is>
       </c>
       <c r="C30" s="1" t="inlineStr">
         <is>
-          <t>UTR187563948837</t>
+          <t>UTR674462208871</t>
         </is>
       </c>
       <c r="D30" s="1" t="inlineStr">
         <is>
-          <t>MERCH_001</t>
+          <t>MERCH_005</t>
         </is>
       </c>
       <c r="E30" s="1" t="n">
-        <v>29909.71</v>
+        <v>19859.55</v>
       </c>
       <c r="F30" s="1" t="n">
-        <v>29909.71</v>
+        <v>19859.55</v>
       </c>
       <c r="G30" s="1" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="H30" s="1" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="I30" s="1" t="n">
@@ -1963,7 +1963,7 @@
       </c>
       <c r="K30" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -1975,12 +1975,12 @@
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
-          <t>pay_631812fbcbd4</t>
+          <t>pay_0d182617af65</t>
         </is>
       </c>
       <c r="C31" s="1" t="inlineStr">
         <is>
-          <t>UTR991885012291</t>
+          <t>UTR700733422645</t>
         </is>
       </c>
       <c r="D31" s="1" t="inlineStr">
@@ -1989,19 +1989,19 @@
         </is>
       </c>
       <c r="E31" s="1" t="n">
-        <v>39718.96</v>
+        <v>15803.1</v>
       </c>
       <c r="F31" s="1" t="n">
-        <v>39718.96</v>
+        <v>15803.1</v>
       </c>
       <c r="G31" s="1" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="H31" s="1" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="I31" s="1" t="n">
@@ -2014,7 +2014,7 @@
       </c>
       <c r="K31" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -2026,33 +2026,33 @@
       </c>
       <c r="B32" s="1" t="inlineStr">
         <is>
-          <t>pay_da30534f3710</t>
+          <t>pay_3868a914262e</t>
         </is>
       </c>
       <c r="C32" s="1" t="inlineStr">
         <is>
-          <t>UTR463415035623</t>
+          <t>UTR33383293041</t>
         </is>
       </c>
       <c r="D32" s="1" t="inlineStr">
         <is>
-          <t>MERCH_004</t>
+          <t>MERCH_001</t>
         </is>
       </c>
       <c r="E32" s="1" t="n">
-        <v>9821.809999999999</v>
+        <v>6964.9</v>
       </c>
       <c r="F32" s="1" t="n">
-        <v>9821.809999999999</v>
+        <v>6964.9</v>
       </c>
       <c r="G32" s="1" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="H32" s="1" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="I32" s="1" t="n">
@@ -2065,7 +2065,7 @@
       </c>
       <c r="K32" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -2077,33 +2077,33 @@
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
-          <t>pay_404870805027</t>
+          <t>pay_1a80b6fed58d</t>
         </is>
       </c>
       <c r="C33" s="1" t="inlineStr">
         <is>
-          <t>UTR779327249932</t>
+          <t>UTR474420383523</t>
         </is>
       </c>
       <c r="D33" s="1" t="inlineStr">
         <is>
-          <t>MERCH_002</t>
+          <t>MERCH_005</t>
         </is>
       </c>
       <c r="E33" s="1" t="n">
-        <v>21396.67</v>
+        <v>16414.02</v>
       </c>
       <c r="F33" s="1" t="n">
-        <v>21396.67</v>
+        <v>16414.02</v>
       </c>
       <c r="G33" s="1" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="H33" s="1" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="I33" s="1" t="n">
@@ -2116,7 +2116,7 @@
       </c>
       <c r="K33" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -2128,33 +2128,33 @@
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
-          <t>pay_9f86181b19dd</t>
+          <t>pay_13680d29187f</t>
         </is>
       </c>
       <c r="C34" s="1" t="inlineStr">
         <is>
-          <t>UTR818500290011</t>
+          <t>UTR969221189477</t>
         </is>
       </c>
       <c r="D34" s="1" t="inlineStr">
         <is>
-          <t>MERCH_003</t>
+          <t>MERCH_004</t>
         </is>
       </c>
       <c r="E34" s="1" t="n">
-        <v>4756.57</v>
+        <v>14034.54</v>
       </c>
       <c r="F34" s="1" t="n">
-        <v>4756.57</v>
+        <v>14034.54</v>
       </c>
       <c r="G34" s="1" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="H34" s="1" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="I34" s="1" t="n">
@@ -2167,7 +2167,7 @@
       </c>
       <c r="K34" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -2179,33 +2179,33 @@
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
-          <t>pay_b7516531808a</t>
+          <t>pay_19b78b7ba3d3</t>
         </is>
       </c>
       <c r="C35" s="1" t="inlineStr">
         <is>
-          <t>UTR460704007312</t>
+          <t>UTR25188744507</t>
         </is>
       </c>
       <c r="D35" s="1" t="inlineStr">
         <is>
-          <t>MERCH_005</t>
+          <t>MERCH_001</t>
         </is>
       </c>
       <c r="E35" s="1" t="n">
-        <v>7608.49</v>
+        <v>16043.46</v>
       </c>
       <c r="F35" s="1" t="n">
-        <v>7608.49</v>
+        <v>16043.46</v>
       </c>
       <c r="G35" s="1" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="H35" s="1" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="I35" s="1" t="n">
@@ -2218,7 +2218,7 @@
       </c>
       <c r="K35" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -2230,33 +2230,33 @@
       </c>
       <c r="B36" s="1" t="inlineStr">
         <is>
-          <t>pay_0ded10d980b1</t>
+          <t>pay_cf1eb80d802c</t>
         </is>
       </c>
       <c r="C36" s="1" t="inlineStr">
         <is>
-          <t>UTR423014459345</t>
+          <t>UTR387403287623</t>
         </is>
       </c>
       <c r="D36" s="1" t="inlineStr">
         <is>
-          <t>MERCH_003</t>
+          <t>MERCH_005</t>
         </is>
       </c>
       <c r="E36" s="1" t="n">
-        <v>17227.44</v>
+        <v>33651.08</v>
       </c>
       <c r="F36" s="1" t="n">
-        <v>17227.44</v>
+        <v>33651.08</v>
       </c>
       <c r="G36" s="1" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="H36" s="1" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I36" s="1" t="n">
@@ -2269,7 +2269,7 @@
       </c>
       <c r="K36" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -2281,33 +2281,33 @@
       </c>
       <c r="B37" s="1" t="inlineStr">
         <is>
-          <t>pay_10cdb4e173ac</t>
+          <t>pay_3d881bb55225</t>
         </is>
       </c>
       <c r="C37" s="1" t="inlineStr">
         <is>
-          <t>UTR543293271401</t>
+          <t>UTR145631941604</t>
         </is>
       </c>
       <c r="D37" s="1" t="inlineStr">
         <is>
-          <t>MERCH_003</t>
+          <t>MERCH_005</t>
         </is>
       </c>
       <c r="E37" s="1" t="n">
-        <v>33952.97</v>
+        <v>35842.89</v>
       </c>
       <c r="F37" s="1" t="n">
-        <v>33952.97</v>
+        <v>35842.89</v>
       </c>
       <c r="G37" s="1" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="H37" s="1" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="I37" s="1" t="n">
@@ -2320,7 +2320,7 @@
       </c>
       <c r="K37" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -2332,33 +2332,33 @@
       </c>
       <c r="B38" s="1" t="inlineStr">
         <is>
-          <t>pay_52b53dce00c5</t>
+          <t>pay_766fbc3dc7f5</t>
         </is>
       </c>
       <c r="C38" s="1" t="inlineStr">
         <is>
-          <t>UTR939869586715</t>
+          <t>UTR857959762051</t>
         </is>
       </c>
       <c r="D38" s="1" t="inlineStr">
         <is>
-          <t>MERCH_002</t>
+          <t>MERCH_004</t>
         </is>
       </c>
       <c r="E38" s="1" t="n">
-        <v>17165.92</v>
+        <v>24949.56</v>
       </c>
       <c r="F38" s="1" t="n">
-        <v>17165.92</v>
+        <v>24949.56</v>
       </c>
       <c r="G38" s="1" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="H38" s="1" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="I38" s="1" t="n">
@@ -2371,7 +2371,7 @@
       </c>
       <c r="K38" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -2383,35 +2383,35 @@
       </c>
       <c r="B39" s="1" t="inlineStr">
         <is>
-          <t>pay_a8309535ff2b</t>
+          <t>pay_3a22f8a1fc63</t>
         </is>
       </c>
       <c r="C39" s="1" t="inlineStr">
         <is>
-          <t>UTR79392417827</t>
+          <t>UTR558875553646</t>
         </is>
       </c>
       <c r="D39" s="1" t="inlineStr">
         <is>
-          <t>MERCH_002</t>
+          <t>MERCH_003</t>
         </is>
       </c>
       <c r="E39" s="1" t="n">
-        <v>34541.17</v>
+        <v>21999.92</v>
       </c>
       <c r="F39" s="1" t="n">
-        <v>34541.17</v>
+        <v>21999.92</v>
       </c>
       <c r="G39" s="1" t="inlineStr">
         <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="H39" s="1" t="inlineStr">
+        <is>
           <t>2026-08-01</t>
         </is>
       </c>
-      <c r="H39" s="1" t="inlineStr">
-        <is>
-          <t>2026-08-03</t>
-        </is>
-      </c>
       <c r="I39" s="1" t="n">
         <v>0.98</v>
       </c>
@@ -2422,7 +2422,7 @@
       </c>
       <c r="K39" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -2434,12 +2434,12 @@
       </c>
       <c r="B40" s="1" t="inlineStr">
         <is>
-          <t>pay_c806891721d5</t>
+          <t>pay_6bd51c1eac40</t>
         </is>
       </c>
       <c r="C40" s="1" t="inlineStr">
         <is>
-          <t>UTR531302577773</t>
+          <t>UTR460662350679</t>
         </is>
       </c>
       <c r="D40" s="1" t="inlineStr">
@@ -2448,19 +2448,19 @@
         </is>
       </c>
       <c r="E40" s="1" t="n">
-        <v>43932.59</v>
+        <v>34279.23</v>
       </c>
       <c r="F40" s="1" t="n">
-        <v>43932.59</v>
+        <v>34279.23</v>
       </c>
       <c r="G40" s="1" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="H40" s="1" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="I40" s="1" t="n">
@@ -2473,7 +2473,7 @@
       </c>
       <c r="K40" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -2485,33 +2485,33 @@
       </c>
       <c r="B41" s="1" t="inlineStr">
         <is>
-          <t>pay_f926b9e36472</t>
+          <t>pay_28dad21f71e1</t>
         </is>
       </c>
       <c r="C41" s="1" t="inlineStr">
         <is>
-          <t>UTR250837499257</t>
+          <t>UTR792378986186</t>
         </is>
       </c>
       <c r="D41" s="1" t="inlineStr">
         <is>
-          <t>MERCH_002</t>
+          <t>MERCH_005</t>
         </is>
       </c>
       <c r="E41" s="1" t="n">
-        <v>38883.58</v>
+        <v>21869.31</v>
       </c>
       <c r="F41" s="1" t="n">
-        <v>38883.58</v>
+        <v>21869.31</v>
       </c>
       <c r="G41" s="1" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="H41" s="1" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="I41" s="1" t="n">
@@ -2524,7 +2524,7 @@
       </c>
       <c r="K41" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -2536,33 +2536,33 @@
       </c>
       <c r="B42" s="1" t="inlineStr">
         <is>
-          <t>pay_2aaebf3811b5</t>
+          <t>pay_63ce8dfc6181</t>
         </is>
       </c>
       <c r="C42" s="1" t="inlineStr">
         <is>
-          <t>UTR88210339955</t>
+          <t>UTR920436609659</t>
         </is>
       </c>
       <c r="D42" s="1" t="inlineStr">
         <is>
-          <t>MERCH_001</t>
+          <t>MERCH_003</t>
         </is>
       </c>
       <c r="E42" s="1" t="n">
-        <v>14860.67</v>
+        <v>17470.05</v>
       </c>
       <c r="F42" s="1" t="n">
-        <v>14860.67</v>
+        <v>17470.05</v>
       </c>
       <c r="G42" s="1" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="H42" s="1" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="I42" s="1" t="n">
@@ -2575,7 +2575,7 @@
       </c>
       <c r="K42" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -2587,33 +2587,33 @@
       </c>
       <c r="B43" s="1" t="inlineStr">
         <is>
-          <t>pay_504671f1f57c</t>
+          <t>pay_9126fdeeeaf8</t>
         </is>
       </c>
       <c r="C43" s="1" t="inlineStr">
         <is>
-          <t>UTR992900378823</t>
+          <t>UTR202516222947</t>
         </is>
       </c>
       <c r="D43" s="1" t="inlineStr">
         <is>
-          <t>MERCH_002</t>
+          <t>MERCH_004</t>
         </is>
       </c>
       <c r="E43" s="1" t="n">
-        <v>22309.36</v>
+        <v>38524.51</v>
       </c>
       <c r="F43" s="1" t="n">
-        <v>22309.36</v>
+        <v>38524.51</v>
       </c>
       <c r="G43" s="1" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="H43" s="1" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="I43" s="1" t="n">
@@ -2626,7 +2626,7 @@
       </c>
       <c r="K43" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -2638,12 +2638,12 @@
       </c>
       <c r="B44" s="1" t="inlineStr">
         <is>
-          <t>pay_737bfe0ee25e</t>
+          <t>pay_f0000a96a081</t>
         </is>
       </c>
       <c r="C44" s="1" t="inlineStr">
         <is>
-          <t>UTR655772731725</t>
+          <t>UTR200311378343</t>
         </is>
       </c>
       <c r="D44" s="1" t="inlineStr">
@@ -2652,14 +2652,14 @@
         </is>
       </c>
       <c r="E44" s="1" t="n">
-        <v>18765.22</v>
+        <v>18489.36</v>
       </c>
       <c r="F44" s="1" t="n">
-        <v>18765.22</v>
+        <v>18489.36</v>
       </c>
       <c r="G44" s="1" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="H44" s="1" t="inlineStr">
@@ -2677,7 +2677,7 @@
       </c>
       <c r="K44" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -2689,33 +2689,33 @@
       </c>
       <c r="B45" s="1" t="inlineStr">
         <is>
-          <t>pay_4d5b3bc2b5d1</t>
+          <t>pay_ed6baf99482b</t>
         </is>
       </c>
       <c r="C45" s="1" t="inlineStr">
         <is>
-          <t>UTR619573524639</t>
+          <t>UTR816031571320</t>
         </is>
       </c>
       <c r="D45" s="1" t="inlineStr">
         <is>
-          <t>MERCH_004</t>
+          <t>MERCH_005</t>
         </is>
       </c>
       <c r="E45" s="1" t="n">
-        <v>888.35</v>
+        <v>11406</v>
       </c>
       <c r="F45" s="1" t="n">
-        <v>888.35</v>
+        <v>11406</v>
       </c>
       <c r="G45" s="1" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="H45" s="1" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="I45" s="1" t="n">
@@ -2728,7 +2728,7 @@
       </c>
       <c r="K45" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -2740,33 +2740,33 @@
       </c>
       <c r="B46" s="1" t="inlineStr">
         <is>
-          <t>pay_ae0f11851350</t>
+          <t>pay_44d72b6b94f1</t>
         </is>
       </c>
       <c r="C46" s="1" t="inlineStr">
         <is>
-          <t>UTR993278379301</t>
+          <t>UTR894885083654</t>
         </is>
       </c>
       <c r="D46" s="1" t="inlineStr">
         <is>
-          <t>MERCH_004</t>
+          <t>MERCH_005</t>
         </is>
       </c>
       <c r="E46" s="1" t="n">
-        <v>2763.45</v>
+        <v>3521.11</v>
       </c>
       <c r="F46" s="1" t="n">
-        <v>2763.45</v>
+        <v>3521.11</v>
       </c>
       <c r="G46" s="1" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="H46" s="1" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="I46" s="1" t="n">
@@ -2779,7 +2779,7 @@
       </c>
       <c r="K46" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -2791,33 +2791,33 @@
       </c>
       <c r="B47" s="1" t="inlineStr">
         <is>
-          <t>pay_7d21b887d326</t>
+          <t>pay_505579f48be6</t>
         </is>
       </c>
       <c r="C47" s="1" t="inlineStr">
         <is>
-          <t>UTR840287359535</t>
+          <t>UTR27185643531</t>
         </is>
       </c>
       <c r="D47" s="1" t="inlineStr">
         <is>
-          <t>MERCH_003</t>
+          <t>MERCH_001</t>
         </is>
       </c>
       <c r="E47" s="1" t="n">
-        <v>42936.15</v>
+        <v>23430.91</v>
       </c>
       <c r="F47" s="1" t="n">
-        <v>42936.15</v>
+        <v>23430.91</v>
       </c>
       <c r="G47" s="1" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="H47" s="1" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="I47" s="1" t="n">
@@ -2830,7 +2830,7 @@
       </c>
       <c r="K47" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -2842,33 +2842,33 @@
       </c>
       <c r="B48" s="1" t="inlineStr">
         <is>
-          <t>pay_5224f1c12d06</t>
+          <t>pay_c4889beb464b</t>
         </is>
       </c>
       <c r="C48" s="1" t="inlineStr">
         <is>
-          <t>UTR867264758101</t>
+          <t>UTR14899803219</t>
         </is>
       </c>
       <c r="D48" s="1" t="inlineStr">
         <is>
-          <t>MERCH_002</t>
+          <t>MERCH_003</t>
         </is>
       </c>
       <c r="E48" s="1" t="n">
-        <v>40792.94</v>
+        <v>33599.2</v>
       </c>
       <c r="F48" s="1" t="n">
-        <v>40792.94</v>
+        <v>33599.2</v>
       </c>
       <c r="G48" s="1" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="H48" s="1" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="I48" s="1" t="n">
@@ -2881,7 +2881,7 @@
       </c>
       <c r="K48" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -2893,33 +2893,33 @@
       </c>
       <c r="B49" s="1" t="inlineStr">
         <is>
-          <t>pay_7fb48821e698</t>
+          <t>pay_9cf6331b1325</t>
         </is>
       </c>
       <c r="C49" s="1" t="inlineStr">
         <is>
-          <t>UTR256138988235</t>
+          <t>UTR619133788282</t>
         </is>
       </c>
       <c r="D49" s="1" t="inlineStr">
         <is>
-          <t>MERCH_005</t>
+          <t>MERCH_004</t>
         </is>
       </c>
       <c r="E49" s="1" t="n">
-        <v>11294.68</v>
+        <v>28328.33</v>
       </c>
       <c r="F49" s="1" t="n">
-        <v>11294.68</v>
+        <v>28328.33</v>
       </c>
       <c r="G49" s="1" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="H49" s="1" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="I49" s="1" t="n">
@@ -2932,7 +2932,7 @@
       </c>
       <c r="K49" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -2944,33 +2944,33 @@
       </c>
       <c r="B50" s="1" t="inlineStr">
         <is>
-          <t>pay_2d1157ce6e05</t>
+          <t>pay_274722deb003</t>
         </is>
       </c>
       <c r="C50" s="1" t="inlineStr">
         <is>
-          <t>UTR285534687363</t>
+          <t>UTR276267968973</t>
         </is>
       </c>
       <c r="D50" s="1" t="inlineStr">
         <is>
-          <t>MERCH_001</t>
+          <t>MERCH_004</t>
         </is>
       </c>
       <c r="E50" s="1" t="n">
-        <v>7915.98</v>
+        <v>13759.74</v>
       </c>
       <c r="F50" s="1" t="n">
-        <v>7915.98</v>
+        <v>13759.74</v>
       </c>
       <c r="G50" s="1" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="H50" s="1" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="I50" s="1" t="n">
@@ -2983,7 +2983,7 @@
       </c>
       <c r="K50" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -2995,33 +2995,33 @@
       </c>
       <c r="B51" s="1" t="inlineStr">
         <is>
-          <t>pay_d4961ff94fc5</t>
+          <t>pay_75fc959978e4</t>
         </is>
       </c>
       <c r="C51" s="1" t="inlineStr">
         <is>
-          <t>UTR715690595534</t>
+          <t>UTR961184942946</t>
         </is>
       </c>
       <c r="D51" s="1" t="inlineStr">
         <is>
-          <t>MERCH_004</t>
+          <t>MERCH_003</t>
         </is>
       </c>
       <c r="E51" s="1" t="n">
-        <v>20361.51</v>
+        <v>15079.71</v>
       </c>
       <c r="F51" s="1" t="n">
-        <v>20361.51</v>
+        <v>15079.71</v>
       </c>
       <c r="G51" s="1" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="H51" s="1" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="I51" s="1" t="n">
@@ -3034,7 +3034,7 @@
       </c>
       <c r="K51" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -3046,33 +3046,33 @@
       </c>
       <c r="B52" s="1" t="inlineStr">
         <is>
-          <t>pay_34b521d1d087</t>
+          <t>pay_cebd133047a7</t>
         </is>
       </c>
       <c r="C52" s="1" t="inlineStr">
         <is>
-          <t>UTR690193133569</t>
+          <t>UTR405078290914</t>
         </is>
       </c>
       <c r="D52" s="1" t="inlineStr">
         <is>
-          <t>MERCH_001</t>
+          <t>MERCH_004</t>
         </is>
       </c>
       <c r="E52" s="1" t="n">
-        <v>2254.5</v>
+        <v>14448</v>
       </c>
       <c r="F52" s="1" t="n">
-        <v>2254.5</v>
+        <v>14448</v>
       </c>
       <c r="G52" s="1" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="H52" s="1" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="I52" s="1" t="n">
@@ -3085,7 +3085,7 @@
       </c>
       <c r="K52" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -3097,33 +3097,33 @@
       </c>
       <c r="B53" s="1" t="inlineStr">
         <is>
-          <t>pay_eaa6933dda63</t>
+          <t>pay_631b4d3304c3</t>
         </is>
       </c>
       <c r="C53" s="1" t="inlineStr">
         <is>
-          <t>UTR126626685338</t>
+          <t>UTR542330883794</t>
         </is>
       </c>
       <c r="D53" s="1" t="inlineStr">
         <is>
-          <t>MERCH_001</t>
+          <t>MERCH_004</t>
         </is>
       </c>
       <c r="E53" s="1" t="n">
-        <v>31256.77</v>
+        <v>36677.2</v>
       </c>
       <c r="F53" s="1" t="n">
-        <v>31256.77</v>
+        <v>36677.2</v>
       </c>
       <c r="G53" s="1" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="H53" s="1" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="I53" s="1" t="n">
@@ -3136,7 +3136,7 @@
       </c>
       <c r="K53" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -3148,33 +3148,33 @@
       </c>
       <c r="B54" s="1" t="inlineStr">
         <is>
-          <t>pay_13ba02e77bef</t>
+          <t>pay_c2d4f8049638</t>
         </is>
       </c>
       <c r="C54" s="1" t="inlineStr">
         <is>
-          <t>UTR714060571995</t>
+          <t>UTR31265224790</t>
         </is>
       </c>
       <c r="D54" s="1" t="inlineStr">
         <is>
-          <t>MERCH_001</t>
+          <t>MERCH_005</t>
         </is>
       </c>
       <c r="E54" s="1" t="n">
-        <v>42084.88</v>
+        <v>22497.52</v>
       </c>
       <c r="F54" s="1" t="n">
-        <v>42084.88</v>
+        <v>22497.52</v>
       </c>
       <c r="G54" s="1" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="H54" s="1" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="I54" s="1" t="n">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="K54" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -3199,33 +3199,33 @@
       </c>
       <c r="B55" s="1" t="inlineStr">
         <is>
-          <t>pay_74701ff14062</t>
+          <t>pay_c86a35f81e08</t>
         </is>
       </c>
       <c r="C55" s="1" t="inlineStr">
         <is>
-          <t>UTR979146404705</t>
+          <t>UTR154116338456</t>
         </is>
       </c>
       <c r="D55" s="1" t="inlineStr">
         <is>
-          <t>MERCH_001</t>
+          <t>MERCH_003</t>
         </is>
       </c>
       <c r="E55" s="1" t="n">
-        <v>21633.2</v>
+        <v>2017.21</v>
       </c>
       <c r="F55" s="1" t="n">
-        <v>21633.2</v>
+        <v>2017.21</v>
       </c>
       <c r="G55" s="1" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="H55" s="1" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="I55" s="1" t="n">
@@ -3238,7 +3238,7 @@
       </c>
       <c r="K55" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -3250,33 +3250,33 @@
       </c>
       <c r="B56" s="1" t="inlineStr">
         <is>
-          <t>pay_68d30c0ab62d</t>
+          <t>pay_c24298090660</t>
         </is>
       </c>
       <c r="C56" s="1" t="inlineStr">
         <is>
-          <t>UTR460808136999</t>
+          <t>UTR501598633425</t>
         </is>
       </c>
       <c r="D56" s="1" t="inlineStr">
         <is>
-          <t>MERCH_005</t>
+          <t>MERCH_001</t>
         </is>
       </c>
       <c r="E56" s="1" t="n">
-        <v>34811.76</v>
+        <v>26811.49</v>
       </c>
       <c r="F56" s="1" t="n">
-        <v>34811.76</v>
+        <v>26811.49</v>
       </c>
       <c r="G56" s="1" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="H56" s="1" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="I56" s="1" t="n">
@@ -3289,7 +3289,7 @@
       </c>
       <c r="K56" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -3301,12 +3301,12 @@
       </c>
       <c r="B57" s="1" t="inlineStr">
         <is>
-          <t>pay_c42c98a5b1d0</t>
+          <t>pay_d042ec97d6f8</t>
         </is>
       </c>
       <c r="C57" s="1" t="inlineStr">
         <is>
-          <t>UTR844298638025</t>
+          <t>UTR119229359780</t>
         </is>
       </c>
       <c r="D57" s="1" t="inlineStr">
@@ -3315,19 +3315,19 @@
         </is>
       </c>
       <c r="E57" s="1" t="n">
-        <v>44422.64</v>
+        <v>44241.42</v>
       </c>
       <c r="F57" s="1" t="n">
-        <v>44422.64</v>
+        <v>44241.42</v>
       </c>
       <c r="G57" s="1" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="H57" s="1" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="I57" s="1" t="n">
@@ -3340,7 +3340,7 @@
       </c>
       <c r="K57" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -3352,33 +3352,33 @@
       </c>
       <c r="B58" s="1" t="inlineStr">
         <is>
-          <t>pay_53d1ca8c4878</t>
+          <t>pay_0390ed2a95f5</t>
         </is>
       </c>
       <c r="C58" s="1" t="inlineStr">
         <is>
-          <t>UTR358185333222</t>
+          <t>UTR434140854000</t>
         </is>
       </c>
       <c r="D58" s="1" t="inlineStr">
         <is>
-          <t>MERCH_002</t>
+          <t>MERCH_004</t>
         </is>
       </c>
       <c r="E58" s="1" t="n">
-        <v>9159.23</v>
+        <v>25608.17</v>
       </c>
       <c r="F58" s="1" t="n">
-        <v>9159.23</v>
+        <v>25608.17</v>
       </c>
       <c r="G58" s="1" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="H58" s="1" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="I58" s="1" t="n">
@@ -3391,7 +3391,7 @@
       </c>
       <c r="K58" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -3403,33 +3403,33 @@
       </c>
       <c r="B59" s="1" t="inlineStr">
         <is>
-          <t>pay_17d8accd6387</t>
+          <t>pay_9e1f11ffdff6</t>
         </is>
       </c>
       <c r="C59" s="1" t="inlineStr">
         <is>
-          <t>UTR335995394883</t>
+          <t>UTR851195759125</t>
         </is>
       </c>
       <c r="D59" s="1" t="inlineStr">
         <is>
-          <t>MERCH_004</t>
+          <t>MERCH_005</t>
         </is>
       </c>
       <c r="E59" s="1" t="n">
-        <v>11030.22</v>
+        <v>40448.48</v>
       </c>
       <c r="F59" s="1" t="n">
-        <v>11030.22</v>
+        <v>40448.48</v>
       </c>
       <c r="G59" s="1" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="H59" s="1" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="I59" s="1" t="n">
@@ -3442,7 +3442,7 @@
       </c>
       <c r="K59" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -3454,33 +3454,33 @@
       </c>
       <c r="B60" s="1" t="inlineStr">
         <is>
-          <t>pay_3167af717ba7</t>
+          <t>pay_94cb2c707957</t>
         </is>
       </c>
       <c r="C60" s="1" t="inlineStr">
         <is>
-          <t>UTR214262047947</t>
+          <t>UTR605918968934</t>
         </is>
       </c>
       <c r="D60" s="1" t="inlineStr">
         <is>
-          <t>MERCH_002</t>
+          <t>MERCH_005</t>
         </is>
       </c>
       <c r="E60" s="1" t="n">
-        <v>6342.39</v>
+        <v>25261.38</v>
       </c>
       <c r="F60" s="1" t="n">
-        <v>6342.39</v>
+        <v>25261.38</v>
       </c>
       <c r="G60" s="1" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="H60" s="1" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="I60" s="1" t="n">
@@ -3493,7 +3493,7 @@
       </c>
       <c r="K60" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -3505,33 +3505,33 @@
       </c>
       <c r="B61" s="1" t="inlineStr">
         <is>
-          <t>pay_159e341e18b7</t>
+          <t>pay_5d784f4e6c93</t>
         </is>
       </c>
       <c r="C61" s="1" t="inlineStr">
         <is>
-          <t>UTR293409590228</t>
+          <t>UTR228101728772</t>
         </is>
       </c>
       <c r="D61" s="1" t="inlineStr">
         <is>
-          <t>MERCH_002</t>
+          <t>MERCH_003</t>
         </is>
       </c>
       <c r="E61" s="1" t="n">
-        <v>19433.31</v>
+        <v>11821.81</v>
       </c>
       <c r="F61" s="1" t="n">
-        <v>19433.31</v>
+        <v>11821.81</v>
       </c>
       <c r="G61" s="1" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="H61" s="1" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="I61" s="1" t="n">
@@ -3544,24 +3544,24 @@
       </c>
       <c r="K61" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="1" t="inlineStr">
         <is>
-          <t>Tier 1 (Exact UTR)</t>
+          <t>Tier 2 (Fuzzy Match)</t>
         </is>
       </c>
       <c r="B62" s="1" t="inlineStr">
         <is>
-          <t>pay_c139c61ee958</t>
+          <t>pay_b39ee5e95ba7</t>
         </is>
       </c>
       <c r="C62" s="1" t="inlineStr">
         <is>
-          <t>UTR457975073557</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D62" s="1" t="inlineStr">
@@ -3570,49 +3570,49 @@
         </is>
       </c>
       <c r="E62" s="1" t="n">
-        <v>29891.22</v>
+        <v>6686.67</v>
       </c>
       <c r="F62" s="1" t="n">
-        <v>29891.22</v>
+        <v>6686.67</v>
       </c>
       <c r="G62" s="1" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="H62" s="1" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="I62" s="1" t="n">
-        <v>0.98</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="J62" s="1" t="inlineStr">
         <is>
-          <t>Exact UTR &amp; Amount Match</t>
+          <t>Fuzzy Match (Amt Var: 0.0, Date Window: T+1)</t>
         </is>
       </c>
       <c r="K62" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="1" t="inlineStr">
         <is>
-          <t>Tier 1 (Exact UTR)</t>
+          <t>Tier 2 (Fuzzy Match)</t>
         </is>
       </c>
       <c r="B63" s="1" t="inlineStr">
         <is>
-          <t>pay_e71be95f11b3</t>
+          <t>pay_2f456ecd203f</t>
         </is>
       </c>
       <c r="C63" s="1" t="inlineStr">
         <is>
-          <t>UTR275156158644</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D63" s="1" t="inlineStr">
@@ -3621,83 +3621,83 @@
         </is>
       </c>
       <c r="E63" s="1" t="n">
-        <v>11967.76</v>
+        <v>20780</v>
       </c>
       <c r="F63" s="1" t="n">
-        <v>11967.76</v>
+        <v>20780</v>
       </c>
       <c r="G63" s="1" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="H63" s="1" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="I63" s="1" t="n">
-        <v>0.98</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="J63" s="1" t="inlineStr">
         <is>
-          <t>Exact UTR &amp; Amount Match</t>
+          <t>Fuzzy Match (Amt Var: 0.0, Date Window: T+2)</t>
         </is>
       </c>
       <c r="K63" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>Tier 1 (Exact UTR)</t>
+          <t>Tier 2 (Fuzzy Match)</t>
         </is>
       </c>
       <c r="B64" s="1" t="inlineStr">
         <is>
-          <t>pay_ea4a2e042d89</t>
+          <t>pay_dacfe3286202</t>
         </is>
       </c>
       <c r="C64" s="1" t="inlineStr">
         <is>
-          <t>UTR692697128543</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D64" s="1" t="inlineStr">
         <is>
-          <t>MERCH_005</t>
+          <t>MERCH_001</t>
         </is>
       </c>
       <c r="E64" s="1" t="n">
-        <v>38980.62</v>
+        <v>2515.53</v>
       </c>
       <c r="F64" s="1" t="n">
-        <v>38980.62</v>
+        <v>2515.53</v>
       </c>
       <c r="G64" s="1" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="H64" s="1" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="I64" s="1" t="n">
-        <v>0.98</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="J64" s="1" t="inlineStr">
         <is>
-          <t>Exact UTR &amp; Amount Match</t>
+          <t>Fuzzy Match (Amt Var: 0.0, Date Window: T+1)</t>
         </is>
       </c>
       <c r="K64" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -3709,33 +3709,33 @@
       </c>
       <c r="B65" s="1" t="inlineStr">
         <is>
-          <t>pay_5a39bb5cde55</t>
+          <t>pay_85898f73e93e</t>
         </is>
       </c>
       <c r="C65" s="1" t="inlineStr">
         <is>
-          <t>UTR540093495457</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D65" s="1" t="inlineStr">
         <is>
-          <t>MERCH_005</t>
+          <t>MERCH_001</t>
         </is>
       </c>
       <c r="E65" s="1" t="n">
-        <v>9880.309999999999</v>
+        <v>1519.67</v>
       </c>
       <c r="F65" s="1" t="n">
-        <v>9880.309999999999</v>
+        <v>1519.67</v>
       </c>
       <c r="G65" s="1" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="H65" s="1" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="I65" s="1" t="n">
@@ -3748,7 +3748,7 @@
       </c>
       <c r="K65" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -3760,7 +3760,7 @@
       </c>
       <c r="B66" s="1" t="inlineStr">
         <is>
-          <t>pay_dfa7939b6c0c</t>
+          <t>pay_f8f1915cb78d</t>
         </is>
       </c>
       <c r="C66" s="1" t="inlineStr">
@@ -3770,23 +3770,23 @@
       </c>
       <c r="D66" s="1" t="inlineStr">
         <is>
-          <t>MERCH_001</t>
+          <t>MERCH_003</t>
         </is>
       </c>
       <c r="E66" s="1" t="n">
-        <v>37534.94</v>
+        <v>18900.85</v>
       </c>
       <c r="F66" s="1" t="n">
-        <v>37534.94</v>
+        <v>18900.85</v>
       </c>
       <c r="G66" s="1" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="H66" s="1" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="I66" s="1" t="n">
@@ -3799,7 +3799,7 @@
       </c>
       <c r="K66" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -3811,33 +3811,33 @@
       </c>
       <c r="B67" s="1" t="inlineStr">
         <is>
-          <t>pay_5000e184e77c</t>
+          <t>pay_4a0a253c1e6e</t>
         </is>
       </c>
       <c r="C67" s="1" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>UTR296578863358</t>
         </is>
       </c>
       <c r="D67" s="1" t="inlineStr">
         <is>
-          <t>MERCH_002</t>
+          <t>MERCH_001</t>
         </is>
       </c>
       <c r="E67" s="1" t="n">
-        <v>23553.07</v>
+        <v>25539.86</v>
       </c>
       <c r="F67" s="1" t="n">
-        <v>23553.07</v>
+        <v>25539.86</v>
       </c>
       <c r="G67" s="1" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="H67" s="1" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="I67" s="1" t="n">
@@ -3850,7 +3850,7 @@
       </c>
       <c r="K67" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -3862,7 +3862,7 @@
       </c>
       <c r="B68" s="1" t="inlineStr">
         <is>
-          <t>pay_a3ce35e8800f</t>
+          <t>pay_072eadf53fd7</t>
         </is>
       </c>
       <c r="C68" s="1" t="inlineStr">
@@ -3872,23 +3872,23 @@
       </c>
       <c r="D68" s="1" t="inlineStr">
         <is>
-          <t>MERCH_001</t>
+          <t>MERCH_004</t>
         </is>
       </c>
       <c r="E68" s="1" t="n">
-        <v>28814.35</v>
+        <v>14936.87</v>
       </c>
       <c r="F68" s="1" t="n">
-        <v>28814.35</v>
+        <v>14936.87</v>
       </c>
       <c r="G68" s="1" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="H68" s="1" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="I68" s="1" t="n">
@@ -3901,7 +3901,7 @@
       </c>
       <c r="K68" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -3913,7 +3913,7 @@
       </c>
       <c r="B69" s="1" t="inlineStr">
         <is>
-          <t>pay_c5b3500b387c</t>
+          <t>pay_af48d54773e8</t>
         </is>
       </c>
       <c r="C69" s="1" t="inlineStr">
@@ -3923,23 +3923,23 @@
       </c>
       <c r="D69" s="1" t="inlineStr">
         <is>
-          <t>MERCH_003</t>
+          <t>MERCH_002</t>
         </is>
       </c>
       <c r="E69" s="1" t="n">
-        <v>15359.69</v>
+        <v>16951.22</v>
       </c>
       <c r="F69" s="1" t="n">
-        <v>15359.69</v>
+        <v>16951.22</v>
       </c>
       <c r="G69" s="1" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="H69" s="1" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="I69" s="1" t="n">
@@ -3952,7 +3952,7 @@
       </c>
       <c r="K69" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -3964,7 +3964,7 @@
       </c>
       <c r="B70" s="1" t="inlineStr">
         <is>
-          <t>pay_fe67fb7174d0</t>
+          <t>pay_1ee2e118f330</t>
         </is>
       </c>
       <c r="C70" s="1" t="inlineStr">
@@ -3978,19 +3978,19 @@
         </is>
       </c>
       <c r="E70" s="1" t="n">
-        <v>44417.91</v>
+        <v>12547.36</v>
       </c>
       <c r="F70" s="1" t="n">
-        <v>44417.91</v>
+        <v>12547.36</v>
       </c>
       <c r="G70" s="1" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="H70" s="1" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="I70" s="1" t="n">
@@ -4003,7 +4003,7 @@
       </c>
       <c r="K70" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -4015,7 +4015,7 @@
       </c>
       <c r="B71" s="1" t="inlineStr">
         <is>
-          <t>pay_e0d6ade423d8</t>
+          <t>pay_3e0bdf2b123f</t>
         </is>
       </c>
       <c r="C71" s="1" t="inlineStr">
@@ -4025,23 +4025,23 @@
       </c>
       <c r="D71" s="1" t="inlineStr">
         <is>
-          <t>MERCH_004</t>
+          <t>MERCH_001</t>
         </is>
       </c>
       <c r="E71" s="1" t="n">
-        <v>35176.73</v>
+        <v>14614.21</v>
       </c>
       <c r="F71" s="1" t="n">
-        <v>35176.73</v>
+        <v>14614.21</v>
       </c>
       <c r="G71" s="1" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="H71" s="1" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="I71" s="1" t="n">
@@ -4049,12 +4049,12 @@
       </c>
       <c r="J71" s="1" t="inlineStr">
         <is>
-          <t>Fuzzy Match (Amt Var: 0.0, Date Window: T+1)</t>
+          <t>Fuzzy Match (Amt Var: 0.0, Date Window: T+2)</t>
         </is>
       </c>
       <c r="K71" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -4066,7 +4066,7 @@
       </c>
       <c r="B72" s="1" t="inlineStr">
         <is>
-          <t>pay_70865b2f5539</t>
+          <t>pay_4adaff422fe3</t>
         </is>
       </c>
       <c r="C72" s="1" t="inlineStr">
@@ -4076,23 +4076,23 @@
       </c>
       <c r="D72" s="1" t="inlineStr">
         <is>
-          <t>MERCH_004</t>
+          <t>MERCH_002</t>
         </is>
       </c>
       <c r="E72" s="1" t="n">
-        <v>14301.39</v>
+        <v>38547.61</v>
       </c>
       <c r="F72" s="1" t="n">
-        <v>14301.39</v>
+        <v>38547.61</v>
       </c>
       <c r="G72" s="1" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="H72" s="1" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="I72" s="1" t="n">
@@ -4100,12 +4100,12 @@
       </c>
       <c r="J72" s="1" t="inlineStr">
         <is>
-          <t>Fuzzy Match (Amt Var: 0.0, Date Window: T+2)</t>
+          <t>Fuzzy Match (Amt Var: 0.0, Date Window: T+1)</t>
         </is>
       </c>
       <c r="K72" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -4117,33 +4117,33 @@
       </c>
       <c r="B73" s="1" t="inlineStr">
         <is>
-          <t>pay_4e603bd00f33</t>
+          <t>pay_9fe3364d60ad</t>
         </is>
       </c>
       <c r="C73" s="1" t="inlineStr">
         <is>
-          <t>UTR815822906509</t>
+          <t>UTR150183464147</t>
         </is>
       </c>
       <c r="D73" s="1" t="inlineStr">
         <is>
-          <t>MERCH_001</t>
+          <t>MERCH_004</t>
         </is>
       </c>
       <c r="E73" s="1" t="n">
-        <v>8527.5</v>
+        <v>25669.78</v>
       </c>
       <c r="F73" s="1" t="n">
-        <v>8527.5</v>
+        <v>25669.78</v>
       </c>
       <c r="G73" s="1" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="H73" s="1" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="I73" s="1" t="n">
@@ -4156,7 +4156,7 @@
       </c>
       <c r="K73" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -4168,7 +4168,7 @@
       </c>
       <c r="B74" s="1" t="inlineStr">
         <is>
-          <t>pay_62b78bdef6b6</t>
+          <t>pay_afe3699bf90a</t>
         </is>
       </c>
       <c r="C74" s="1" t="inlineStr">
@@ -4178,23 +4178,23 @@
       </c>
       <c r="D74" s="1" t="inlineStr">
         <is>
-          <t>MERCH_001</t>
+          <t>MERCH_002</t>
         </is>
       </c>
       <c r="E74" s="1" t="n">
-        <v>5140.68</v>
+        <v>32771.99</v>
       </c>
       <c r="F74" s="1" t="n">
-        <v>5140.68</v>
+        <v>32771.99</v>
       </c>
       <c r="G74" s="1" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="H74" s="1" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="I74" s="1" t="n">
@@ -4202,12 +4202,12 @@
       </c>
       <c r="J74" s="1" t="inlineStr">
         <is>
-          <t>Fuzzy Match (Amt Var: 0.0, Date Window: T+1)</t>
+          <t>Fuzzy Match (Amt Var: 0.0, Date Window: T+2)</t>
         </is>
       </c>
       <c r="K74" s="1" t="inlineStr">
         <is>
-          <t>2026-08-26 19:40:42</t>
+          <t>2026-08-26 19:54:28</t>
         </is>
       </c>
     </row>
@@ -4222,7 +4222,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N24"/>
+  <dimension ref="A1:N18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4305,25 +4305,25 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>bank_TXN5944760984</t>
+          <t>bank_TXN5185222750</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>UTR540093495457</t>
+          <t>UTR150183464147</t>
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>9880.309999999999</v>
+        <v>25669.78</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>MERCH_005</t>
+          <t>MERCH_004</t>
         </is>
       </c>
       <c r="G2" s="2" t="n">
@@ -4331,7 +4331,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Duplicate transaction detected for UTR UTR540093495457 (₹9,880.31). Multiple credits registered in bank statement for a single settlement item.</t>
+          <t>Duplicate transaction detected for UTR UTR150183464147 (₹25,669.78). Multiple credits registered in bank statement for a single settlement item.</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -4353,20 +4353,20 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>bank_TXN5311549960</t>
+          <t>bank_TXN1359561754</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>UTR815822906509</t>
+          <t>UTR296578863358</t>
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>8527.5</v>
+        <v>25539.86</v>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -4379,7 +4379,7 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Duplicate transaction detected for UTR UTR815822906509 (₹8,527.50). Multiple credits registered in bank statement for a single settlement item.</t>
+          <t>Duplicate transaction detected for UTR UTR296578863358 (₹25,539.86). Multiple credits registered in bank statement for a single settlement item.</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
@@ -4396,25 +4396,21 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Amount Mismatch</t>
+          <t>Timing Mismatch</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>pay_f535fef2f1fb</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>UTR158868713572</t>
-        </is>
-      </c>
+          <t>pay_bb157f491fec</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr"/>
       <c r="D4" s="2" t="n">
-        <v>39058.05</v>
+        <v>17434.98</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -4423,32 +4419,32 @@
         </is>
       </c>
       <c r="G4" s="2" t="n">
-        <v>0.89</v>
+        <v>0.92</v>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Razorpay settled ₹39,058.05 on 2026-08-14, but bank credited ₹37,886.31 (diff of ₹1,171.74 or 3.0%). Likely caused by MDR tier rate shift or pending refund adjustment.</t>
+          <t>Payment pay_bb157f491fec (₹17,434.98) settled on 2026-08-10 in Razorpay, but bank credited on 2026-08-16 (&gt;3 day gap). Overlap with weekend/bank holiday detected.</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Verify MDR fee rate schedule in Razorpay dashboard and check for unadjusted chargeback fees.</t>
+          <t>Wait for T+3 clearance cycle to complete or verify RBI Nodal bank settlement schedule.</t>
         </is>
       </c>
       <c r="J4" s="2" t="n">
-        <v>39058.05</v>
+        <v>17434.98</v>
       </c>
       <c r="K4" s="2" t="n">
-        <v>37886.31</v>
+        <v>17434.98</v>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr"/>
@@ -4456,73 +4452,81 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Missing Entry (Bank)</t>
+          <t>Amount Mismatch</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>pay_204d68b0a894</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>UTR794741895767</t>
-        </is>
-      </c>
+          <t>pay_0aac44477c64</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr"/>
       <c r="D5" s="2" t="n">
-        <v>35966.94</v>
+        <v>19095.55</v>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>MERCH_005</t>
+          <t>MERCH_004</t>
         </is>
       </c>
       <c r="G5" s="2" t="n">
-        <v>0.88</v>
+        <v>0.89</v>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Razorpay payment pay_204d68b0a894 (₹35,966.94) processed on 2026-08-21 shows status 'settled', but no corresponding credit is reflected in bank statement within T+3 window.</t>
+          <t>Razorpay settled ₹19,095.55 on 2026-08-01, but bank credited ₹19,859.37 (diff of ₹763.82 or 4.0%). Likely caused by MDR tier rate shift or pending refund adjustment.</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Check nodal bank reference number (UTR) with acquiring bank or request Razorpay support trace.</t>
-        </is>
-      </c>
-      <c r="J5" s="2" t="inlineStr"/>
-      <c r="K5" s="2" t="inlineStr"/>
-      <c r="L5" s="2" t="inlineStr"/>
-      <c r="M5" s="2" t="inlineStr"/>
+          <t>Verify MDR fee rate schedule in Razorpay dashboard and check for unadjusted chargeback fees.</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="n">
+        <v>19095.55</v>
+      </c>
+      <c r="K5" s="2" t="n">
+        <v>19859.37</v>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
       <c r="N5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Amount Mismatch</t>
+          <t>Missing Entry (Bank)</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>pay_8335d0243885</t>
+          <t>pay_7734663dee65</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>UTR170810869649</t>
+          <t>UTR383100665216</t>
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>20984.03</v>
+        <v>3466.74</v>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -4531,88 +4535,80 @@
         </is>
       </c>
       <c r="G6" s="2" t="n">
-        <v>0.89</v>
+        <v>0.88</v>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Razorpay settled ₹20,984.03 on 2026-08-17, but bank credited ₹37,886.31 (diff of ₹16,902.28 or 80.5%). Likely caused by MDR tier rate shift or pending refund adjustment.</t>
+          <t>Razorpay payment pay_7734663dee65 (₹3,466.74) processed on 2026-07-29 shows status 'settled', but no corresponding credit is reflected in bank statement within T+3 window.</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Verify MDR fee rate schedule in Razorpay dashboard and check for unadjusted chargeback fees.</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="n">
-        <v>20984.03</v>
-      </c>
-      <c r="K6" s="2" t="n">
-        <v>37886.31</v>
-      </c>
-      <c r="L6" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-17</t>
-        </is>
-      </c>
-      <c r="M6" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-15</t>
-        </is>
-      </c>
+          <t>Check nodal bank reference number (UTR) with acquiring bank or request Razorpay support trace.</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr"/>
+      <c r="K6" s="2" t="inlineStr"/>
+      <c r="L6" s="2" t="inlineStr"/>
+      <c r="M6" s="2" t="inlineStr"/>
       <c r="N6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Timing Mismatch</t>
+          <t>Amount Mismatch</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>pay_bcec812e60a7</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr"/>
+          <t>pay_ab65e3b3de66</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>UTR554865232848</t>
+        </is>
+      </c>
       <c r="D7" s="2" t="n">
-        <v>39515.84</v>
+        <v>9573.879999999999</v>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>MERCH_003</t>
+          <t>MERCH_001</t>
         </is>
       </c>
       <c r="G7" s="2" t="n">
-        <v>0.92</v>
+        <v>0.89</v>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Payment pay_bcec812e60a7 (₹39,515.84) settled on 2026-07-28 in Razorpay, but bank credited on 2026-08-02 (&gt;3 day gap). Overlap with weekend/bank holiday detected.</t>
+          <t>Razorpay settled ₹9,573.88 on 2026-07-31, but bank credited ₹25,539.86 (diff of ₹15,965.98 or 166.8%). Likely caused by MDR tier rate shift or pending refund adjustment.</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>Wait for T+3 clearance cycle to complete or verify RBI Nodal bank settlement schedule.</t>
+          <t>Verify MDR fee rate schedule in Razorpay dashboard and check for unadjusted chargeback fees.</t>
         </is>
       </c>
       <c r="J7" s="2" t="n">
-        <v>39515.84</v>
+        <v>9573.879999999999</v>
       </c>
       <c r="K7" s="2" t="n">
-        <v>39515.84</v>
+        <v>25539.86</v>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr"/>
@@ -4625,25 +4621,25 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>pay_17460bdd50be</t>
+          <t>pay_f50054af5679</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>UTR490880138910</t>
+          <t>UTR11116946832</t>
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>36925.38</v>
+        <v>18118.44</v>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>MERCH_003</t>
+          <t>MERCH_004</t>
         </is>
       </c>
       <c r="G8" s="2" t="n">
@@ -4651,7 +4647,7 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Razorpay settled ₹36,925.38 on 2026-07-27, but bank credited ₹35,817.62 (diff of ₹1,107.76 or 3.0%). Likely caused by MDR tier rate shift or pending refund adjustment.</t>
+          <t>Razorpay settled ₹18,118.44 on 2026-08-20, but bank credited ₹25,669.78 (diff of ₹7,551.34 or 41.7%). Likely caused by MDR tier rate shift or pending refund adjustment.</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
@@ -4660,19 +4656,19 @@
         </is>
       </c>
       <c r="J8" s="2" t="n">
-        <v>36925.38</v>
+        <v>18118.44</v>
       </c>
       <c r="K8" s="2" t="n">
-        <v>35817.62</v>
+        <v>25669.78</v>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr"/>
@@ -4685,20 +4681,20 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>pay_9a2324e90653</t>
+          <t>pay_bae5691909a2</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>UTR20229858812</t>
+          <t>UTR1010556463</t>
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>22527.15</v>
+        <v>36857.36</v>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -4711,7 +4707,7 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Razorpay payment pay_9a2324e90653 (₹22,527.15) processed on 2026-08-19 shows status 'settled', but no corresponding credit is reflected in bank statement within T+3 window.</t>
+          <t>Razorpay payment pay_bae5691909a2 (₹36,857.36) processed on 2026-08-03 shows status 'settled', but no corresponding credit is reflected in bank statement within T+3 window.</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
@@ -4733,20 +4729,20 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>pay_2820ac589747</t>
+          <t>pay_cd1129d6d189</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>UTR151866570063</t>
+          <t>UTR891847135336</t>
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>32216.18</v>
+        <v>15625.65</v>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -4759,7 +4755,7 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Razorpay settled ₹32,216.18 on 2026-08-15, but bank credited ₹8,527.50 (diff of ₹23,688.68 or 73.5%). Likely caused by MDR tier rate shift or pending refund adjustment.</t>
+          <t>Razorpay settled ₹15,625.65 on 2026-08-16, but bank credited ₹15,156.88 (diff of ₹468.77 or 3.0%). Likely caused by MDR tier rate shift or pending refund adjustment.</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
@@ -4768,14 +4764,14 @@
         </is>
       </c>
       <c r="J10" s="2" t="n">
-        <v>32216.18</v>
+        <v>15625.65</v>
       </c>
       <c r="K10" s="2" t="n">
-        <v>8527.5</v>
+        <v>15156.88</v>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
@@ -4793,20 +4789,16 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>unlinked_TXN9725288329</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>UTR158868713572</t>
-        </is>
-      </c>
+          <t>unlinked_TXN6225041573</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr"/>
       <c r="D11" s="2" t="n">
-        <v>37886.31</v>
+        <v>17434.98</v>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -4819,7 +4811,7 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Bank received credit of ₹37,886.31 on 2026-08-15 with narration 'TXN9725288329', but no matching settlement record exists in Razorpay sandbox API.</t>
+          <t>Bank received credit of ₹17,434.98 on 2026-08-16 with narration 'TXN6225041573', but no matching settlement record exists in Razorpay sandbox API.</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
@@ -4833,7 +4825,7 @@
       <c r="M11" s="2" t="inlineStr"/>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>TXN9725288329</t>
+          <t>TXN6225041573</t>
         </is>
       </c>
     </row>
@@ -4845,25 +4837,21 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>unlinked_TXN8115872962</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>UTR170810869649</t>
-        </is>
-      </c>
+          <t>unlinked_TXN3535692117</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr"/>
       <c r="D12" s="2" t="n">
-        <v>21823.39</v>
+        <v>19859.37</v>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>MERCH_003</t>
+          <t>MERCH_004</t>
         </is>
       </c>
       <c r="G12" s="2" t="n">
@@ -4871,7 +4859,7 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Bank received credit of ₹21,823.39 on 2026-08-18 with narration 'TXN8115872962', but no matching settlement record exists in Razorpay sandbox API.</t>
+          <t>Bank received credit of ₹19,859.37 on 2026-08-02 with narration 'TXN3535692117', but no matching settlement record exists in Razorpay sandbox API.</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
@@ -4885,7 +4873,7 @@
       <c r="M12" s="2" t="inlineStr"/>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>TXN8115872962</t>
+          <t>TXN3535692117</t>
         </is>
       </c>
     </row>
@@ -4897,21 +4885,25 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>unlinked_TXN3920817145</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr"/>
+          <t>unlinked_TXN2597998601</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>UTR891847135336</t>
+        </is>
+      </c>
       <c r="D13" s="2" t="n">
-        <v>39515.84</v>
+        <v>15156.88</v>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>MERCH_003</t>
+          <t>MERCH_001</t>
         </is>
       </c>
       <c r="G13" s="2" t="n">
@@ -4919,7 +4911,7 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>Bank received credit of ₹39,515.84 on 2026-08-02 with narration 'TXN3920817145', but no matching settlement record exists in Razorpay sandbox API.</t>
+          <t>Bank received credit of ₹15,156.88 on 2026-08-17 with narration 'TXN2597998601', but no matching settlement record exists in Razorpay sandbox API.</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
@@ -4933,7 +4925,7 @@
       <c r="M13" s="2" t="inlineStr"/>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>TXN3920817145</t>
+          <t>TXN2597998601</t>
         </is>
       </c>
     </row>
@@ -4945,25 +4937,25 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>unlinked_TXN4480551152</t>
+          <t>unlinked_TXN6052322294</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>UTR490880138910</t>
+          <t>UTR651959637639</t>
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>35817.62</v>
+        <v>13673.02</v>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>MERCH_003</t>
+          <t>MERCH_005</t>
         </is>
       </c>
       <c r="G14" s="2" t="n">
@@ -4971,7 +4963,7 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Bank received credit of ₹35,817.62 on 2026-07-28 with narration 'TXN4480551152', but no matching settlement record exists in Razorpay sandbox API.</t>
+          <t>Bank received credit of ₹13,673.02 on 2026-08-09 with narration 'TXN6052322294', but no matching settlement record exists in Razorpay sandbox API.</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
@@ -4985,7 +4977,7 @@
       <c r="M14" s="2" t="inlineStr"/>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>TXN4480551152</t>
+          <t>TXN6052322294</t>
         </is>
       </c>
     </row>
@@ -4997,25 +4989,25 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>unlinked_TXN9943392397</t>
+          <t>unlinked_TXN6162382030</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>UTR151866570063</t>
+          <t>UTR936192221913</t>
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>33182.67</v>
+        <v>5786.38</v>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>MERCH_001</t>
+          <t>MERCH_005</t>
         </is>
       </c>
       <c r="G15" s="2" t="n">
@@ -5023,7 +5015,7 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>Bank received credit of ₹33,182.67 on 2026-08-16 with narration 'TXN9943392397', but no matching settlement record exists in Razorpay sandbox API.</t>
+          <t>Bank received credit of ₹5,786.38 on 2026-08-20 with narration 'TXN6162382030', but no matching settlement record exists in Razorpay sandbox API.</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
@@ -5037,7 +5029,7 @@
       <c r="M15" s="2" t="inlineStr"/>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>TXN9943392397</t>
+          <t>TXN6162382030</t>
         </is>
       </c>
     </row>
@@ -5049,16 +5041,16 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>unlinked_TXN1345783029</t>
+          <t>unlinked_TXN1390112004</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>UTR840955633250</t>
+          <t>UTR622941429654</t>
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>13488.29</v>
+        <v>5252.53</v>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
@@ -5067,7 +5059,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>MERCH_002</t>
+          <t>MERCH_004</t>
         </is>
       </c>
       <c r="G16" s="2" t="n">
@@ -5075,7 +5067,7 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Bank received credit of ₹13,488.29 on 2026-08-12 with narration 'TXN1345783029', but no matching settlement record exists in Razorpay sandbox API.</t>
+          <t>Bank received credit of ₹5,252.53 on 2026-08-12 with narration 'TXN1390112004', but no matching settlement record exists in Razorpay sandbox API.</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
@@ -5089,377 +5081,97 @@
       <c r="M16" s="2" t="inlineStr"/>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>TXN1345783029</t>
+          <t>TXN1390112004</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Missing Entry (Razorpay)</t>
+          <t>GST Variance</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>unlinked_TXN1439843164</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>UTR545774621770</t>
-        </is>
-      </c>
+          <t>pay_766fbc3dc7f5</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr"/>
       <c r="D17" s="2" t="n">
-        <v>8276.200000000001</v>
+        <v>25520.44</v>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>MERCH_002</t>
+          <t>MERCH_004</t>
         </is>
       </c>
       <c r="G17" s="2" t="n">
-        <v>0.85</v>
+        <v>0.91</v>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>Bank received credit of ₹8,276.20 on 2026-08-10 with narration 'TXN1439843164', but no matching settlement record exists in Razorpay sandbox API.</t>
+          <t>GST calculation variance detected on transaction pay_766fbc3dc7f5 (₹25,520.44). Calculated GST on MDR differs from GST return filing.</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>Verify if payment was received directly via offline UPI QR or secondary payment gateway.</t>
+          <t>Reconcile GSTR-2B input tax credit entries against Razorpay monthly GST tax invoices.</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr"/>
       <c r="K17" s="2" t="inlineStr"/>
       <c r="L17" s="2" t="inlineStr"/>
       <c r="M17" s="2" t="inlineStr"/>
-      <c r="N17" s="2" t="inlineStr">
-        <is>
-          <t>TXN1439843164</t>
-        </is>
-      </c>
+      <c r="N17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Missing Entry (Razorpay)</t>
+          <t>GST Variance</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>unlinked_TXN6367528777</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>UTR277447427560</t>
-        </is>
-      </c>
+          <t>pay_d042ec97d6f8</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr"/>
       <c r="D18" s="2" t="n">
-        <v>6896.62</v>
+        <v>45253.72</v>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>MERCH_003</t>
+          <t>MERCH_005</t>
         </is>
       </c>
       <c r="G18" s="2" t="n">
-        <v>0.85</v>
+        <v>0.91</v>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Bank received credit of ₹6,896.62 on 2026-08-07 with narration 'TXN6367528777', but no matching settlement record exists in Razorpay sandbox API.</t>
+          <t>GST calculation variance detected on transaction pay_d042ec97d6f8 (₹45,253.72). Calculated GST on MDR differs from GST return filing.</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>Verify if payment was received directly via offline UPI QR or secondary payment gateway.</t>
+          <t>Reconcile GSTR-2B input tax credit entries against Razorpay monthly GST tax invoices.</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr"/>
       <c r="K18" s="2" t="inlineStr"/>
       <c r="L18" s="2" t="inlineStr"/>
       <c r="M18" s="2" t="inlineStr"/>
-      <c r="N18" s="2" t="inlineStr">
-        <is>
-          <t>TXN6367528777</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>GST Variance</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>pay_cf92979f2c52</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr"/>
-      <c r="D19" s="2" t="n">
-        <v>3973.61</v>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-18</t>
-        </is>
-      </c>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>MERCH_001</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="n">
-        <v>0.91</v>
-      </c>
-      <c r="H19" s="2" t="inlineStr">
-        <is>
-          <t>GST calculation variance detected on transaction pay_cf92979f2c52 (₹3,973.61). Calculated GST on MDR differs from GST return filing.</t>
-        </is>
-      </c>
-      <c r="I19" s="2" t="inlineStr">
-        <is>
-          <t>Reconcile GSTR-2B input tax credit entries against Razorpay monthly GST tax invoices.</t>
-        </is>
-      </c>
-      <c r="J19" s="2" t="inlineStr"/>
-      <c r="K19" s="2" t="inlineStr"/>
-      <c r="L19" s="2" t="inlineStr"/>
-      <c r="M19" s="2" t="inlineStr"/>
-      <c r="N19" s="2" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>GST Variance</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>pay_504671f1f57c</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr"/>
-      <c r="D20" s="2" t="n">
-        <v>21798.89</v>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-30</t>
-        </is>
-      </c>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>MERCH_002</t>
-        </is>
-      </c>
-      <c r="G20" s="2" t="n">
-        <v>0.91</v>
-      </c>
-      <c r="H20" s="2" t="inlineStr">
-        <is>
-          <t>GST calculation variance detected on transaction pay_504671f1f57c (₹21,798.89). Calculated GST on MDR differs from GST return filing.</t>
-        </is>
-      </c>
-      <c r="I20" s="2" t="inlineStr">
-        <is>
-          <t>Reconcile GSTR-2B input tax credit entries against Razorpay monthly GST tax invoices.</t>
-        </is>
-      </c>
-      <c r="J20" s="2" t="inlineStr"/>
-      <c r="K20" s="2" t="inlineStr"/>
-      <c r="L20" s="2" t="inlineStr"/>
-      <c r="M20" s="2" t="inlineStr"/>
-      <c r="N20" s="2" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>GST Variance</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>pay_34b521d1d087</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr"/>
-      <c r="D21" s="2" t="n">
-        <v>2202.91</v>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-09</t>
-        </is>
-      </c>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>MERCH_001</t>
-        </is>
-      </c>
-      <c r="G21" s="2" t="n">
-        <v>0.91</v>
-      </c>
-      <c r="H21" s="2" t="inlineStr">
-        <is>
-          <t>GST calculation variance detected on transaction pay_34b521d1d087 (₹2,202.91). Calculated GST on MDR differs from GST return filing.</t>
-        </is>
-      </c>
-      <c r="I21" s="2" t="inlineStr">
-        <is>
-          <t>Reconcile GSTR-2B input tax credit entries against Razorpay monthly GST tax invoices.</t>
-        </is>
-      </c>
-      <c r="J21" s="2" t="inlineStr"/>
-      <c r="K21" s="2" t="inlineStr"/>
-      <c r="L21" s="2" t="inlineStr"/>
-      <c r="M21" s="2" t="inlineStr"/>
-      <c r="N21" s="2" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>GST Variance</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>pay_e0d6ade423d8</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr"/>
-      <c r="D22" s="2" t="n">
-        <v>34371.84</v>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-08</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>MERCH_004</t>
-        </is>
-      </c>
-      <c r="G22" s="2" t="n">
-        <v>0.91</v>
-      </c>
-      <c r="H22" s="2" t="inlineStr">
-        <is>
-          <t>GST calculation variance detected on transaction pay_e0d6ade423d8 (₹34,371.84). Calculated GST on MDR differs from GST return filing.</t>
-        </is>
-      </c>
-      <c r="I22" s="2" t="inlineStr">
-        <is>
-          <t>Reconcile GSTR-2B input tax credit entries against Razorpay monthly GST tax invoices.</t>
-        </is>
-      </c>
-      <c r="J22" s="2" t="inlineStr"/>
-      <c r="K22" s="2" t="inlineStr"/>
-      <c r="L22" s="2" t="inlineStr"/>
-      <c r="M22" s="2" t="inlineStr"/>
-      <c r="N22" s="2" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>GST Variance</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>pay_53d1ca8c4878</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="inlineStr"/>
-      <c r="D23" s="2" t="n">
-        <v>9368.809999999999</v>
-      </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-06</t>
-        </is>
-      </c>
-      <c r="F23" s="2" t="inlineStr">
-        <is>
-          <t>MERCH_002</t>
-        </is>
-      </c>
-      <c r="G23" s="2" t="n">
-        <v>0.91</v>
-      </c>
-      <c r="H23" s="2" t="inlineStr">
-        <is>
-          <t>GST calculation variance detected on transaction pay_53d1ca8c4878 (₹9,368.81). Calculated GST on MDR differs from GST return filing.</t>
-        </is>
-      </c>
-      <c r="I23" s="2" t="inlineStr">
-        <is>
-          <t>Reconcile GSTR-2B input tax credit entries against Razorpay monthly GST tax invoices.</t>
-        </is>
-      </c>
-      <c r="J23" s="2" t="inlineStr"/>
-      <c r="K23" s="2" t="inlineStr"/>
-      <c r="L23" s="2" t="inlineStr"/>
-      <c r="M23" s="2" t="inlineStr"/>
-      <c r="N23" s="2" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>GST Variance</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>pay_ea4a2e042d89</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr"/>
-      <c r="D24" s="2" t="n">
-        <v>39872.55</v>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-27</t>
-        </is>
-      </c>
-      <c r="F24" s="2" t="inlineStr">
-        <is>
-          <t>MERCH_005</t>
-        </is>
-      </c>
-      <c r="G24" s="2" t="n">
-        <v>0.91</v>
-      </c>
-      <c r="H24" s="2" t="inlineStr">
-        <is>
-          <t>GST calculation variance detected on transaction pay_ea4a2e042d89 (₹39,872.55). Calculated GST on MDR differs from GST return filing.</t>
-        </is>
-      </c>
-      <c r="I24" s="2" t="inlineStr">
-        <is>
-          <t>Reconcile GSTR-2B input tax credit entries against Razorpay monthly GST tax invoices.</t>
-        </is>
-      </c>
-      <c r="J24" s="2" t="inlineStr"/>
-      <c r="K24" s="2" t="inlineStr"/>
-      <c r="L24" s="2" t="inlineStr"/>
-      <c r="M24" s="2" t="inlineStr"/>
-      <c r="N24" s="2" t="inlineStr"/>
+      <c r="N18" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>